<commit_message>
MB001 #327: separate disputed debt and verify printable reconciliation candidate
</commit_message>
<xml_diff>
--- a/tools/candidates/s1-oplata-za-raboty/02-proverka-i-kontrol-otveta.xlsx
+++ b/tools/candidates/s1-oplata-za-raboty/02-proverka-i-kontrol-otveta.xlsx
@@ -799,7 +799,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="123" customHeight="1">
+    <row r="24" ht="153" customHeight="1">
       <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Следующий шаг</t>
@@ -5195,7 +5195,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Внесите каждую операцию в реестр взаиморасчётов с типом «Удержание», «Зачёт» или «Неустойка заявлена». Бесспорную часть долга можно вести по S1 дальше; спорную часть с документами передайте специалисту до направления претензии.</t>
+          <t>Внесите каждую операцию в файл 04, лист «Взаиморасчёты», с типом «Удержание», «Зачёт встречного требования» или «Неустойка заявлена» и с актом, к которому она относится. Общий долг она не уменьшает: её сумма показывается отдельно как спорная часть. В расчёт процентов и претензию идёт только бесспорная часть — её можно вести по S1 дальше; спорную часть с документами передайте специалисту до направления претензии.</t>
         </is>
       </c>
     </row>
@@ -5212,7 +5212,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Суммы по допработам, которые заказчик не подписал, не вносите в реестр взаиморасчётов как начисление по акту: эти работы не приняты. Если допработы вошли в подписанный акт, эта часть долга спорная: в расчёт процентов и претензию её без оценки специалиста не включайте. Бесспорную часть долга ведите по маршруту дальше. По допработам соберите договор, смету, переписку о поручении работ и акты и передайте специалисту по описи (файл 10, раздел В).</t>
+          <t>Суммы по допработам, которые заказчик не подписал, не вносите в реестр взаиморасчётов как начисление по акту: эти работы не приняты. Если допработы вошли в подписанный акт, эта часть долга спорная: внесите её в файл 04, лист «Взаиморасчёты», операцией «Допработы без соглашения (спорно)» с актом — она попадёт в спорную часть и в расчёт процентов и претензию без оценки специалиста не войдёт. Бесспорную часть долга ведите по маршруту дальше. По допработам соберите договор, смету, переписку о поручении работ и акты и передайте специалисту по описи (файл 10, раздел В).</t>
         </is>
       </c>
     </row>

</xml_diff>